<commit_message>
Working on methods and results sections of paper
</commit_message>
<xml_diff>
--- a/Tables/MAIHDA.xlsx
+++ b/Tables/MAIHDA.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/38b97e870d12de33/Documents/UAH/PhD Documents/INEdatos/Analysis/Tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{980E5B5A-75EE-4430-85D2-0D88ED2233B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C3DFA13-7A7B-47D9-BAE2-828DB4EFF82F}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{980E5B5A-75EE-4430-85D2-0D88ED2233B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0FCB3D0-F854-4808-B0F0-93B503ECB1CF}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1572" yWindow="3804" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{F53BC189-169C-4D5A-95F0-57F331A1907F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F53BC189-169C-4D5A-95F0-57F331A1907F}"/>
   </bookViews>
   <sheets>
     <sheet name="MAIHDA-0412" sheetId="1" r:id="rId1"/>
-    <sheet name="MAIHDA (2)" sheetId="2" r:id="rId2"/>
-    <sheet name="MAIHDA" sheetId="3" r:id="rId3"/>
+    <sheet name="MAIHDA (2)" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="MAIHDA" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1312,57 +1312,6 @@
     <xf numFmtId="164" fontId="2" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1378,6 +1327,57 @@
     </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1669,14 +1669,17 @@
     <col min="4" max="4" width="15.5546875" style="1" customWidth="1"/>
     <col min="5" max="6" width="9.109375" style="1"/>
     <col min="7" max="7" width="14.88671875" style="1" customWidth="1"/>
-    <col min="8" max="9" width="9.109375" style="1"/>
+    <col min="8" max="8" width="6.109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="9.109375" style="1"/>
     <col min="10" max="10" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="9.109375" style="1"/>
-    <col min="15" max="15" width="11.44140625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="13.109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="18.88671875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="7" style="1" customWidth="1"/>
+    <col min="13" max="13" width="8" style="1" customWidth="1"/>
+    <col min="14" max="14" width="6.6640625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="10.77734375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="12" style="1" customWidth="1"/>
     <col min="17" max="17" width="10" style="1" customWidth="1"/>
-    <col min="18" max="18" width="19.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="13" style="1" customWidth="1"/>
     <col min="20" max="21" width="9.109375" style="1"/>
     <col min="22" max="22" width="29.88671875" style="1" bestFit="1" customWidth="1"/>
@@ -1747,18 +1750,18 @@
     </row>
     <row r="9" spans="1:11" ht="28.2" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
-      <c r="B9" s="50" t="s">
+      <c r="B9" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="50"/>
-      <c r="D9" s="50"/>
+      <c r="C9" s="44"/>
+      <c r="D9" s="44"/>
       <c r="G9" s="3"/>
-      <c r="H9" s="50" t="s">
+      <c r="H9" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="I9" s="50"/>
-      <c r="J9" s="50"/>
-      <c r="K9" s="50"/>
+      <c r="I9" s="44"/>
+      <c r="J9" s="44"/>
+      <c r="K9" s="44"/>
     </row>
     <row r="10" spans="1:11" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
@@ -1819,12 +1822,12 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
+      <c r="B12" s="45"/>
+      <c r="C12" s="45"/>
+      <c r="D12" s="45"/>
       <c r="G12" s="6" t="s">
         <v>19</v>
       </c>
@@ -1845,11 +1848,11 @@
       <c r="A13" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="46">
+      <c r="B13" s="41">
         <v>3.29</v>
       </c>
-      <c r="C13" s="46"/>
-      <c r="D13" s="46"/>
+      <c r="C13" s="41"/>
+      <c r="D13" s="41"/>
       <c r="G13" s="6" t="s">
         <v>22</v>
       </c>
@@ -1870,11 +1873,11 @@
       <c r="A14" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="46">
+      <c r="B14" s="41">
         <v>0.28000000000000003</v>
       </c>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
+      <c r="C14" s="41"/>
+      <c r="D14" s="41"/>
       <c r="G14" s="6" t="s">
         <v>25</v>
       </c>
@@ -1895,24 +1898,24 @@
       <c r="A15" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="46">
+      <c r="B15" s="41">
         <v>0.08</v>
       </c>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="41"/>
       <c r="G15" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="H15" s="38">
+      <c r="H15" s="42">
         <v>0.62</v>
       </c>
-      <c r="I15" s="38">
+      <c r="I15" s="42">
         <v>0.04</v>
       </c>
-      <c r="J15" s="38" t="s">
+      <c r="J15" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="K15" s="51" t="s">
+      <c r="K15" s="43" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1920,28 +1923,28 @@
       <c r="A16" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="44">
+      <c r="B16" s="49">
         <v>72</v>
       </c>
-      <c r="C16" s="44"/>
-      <c r="D16" s="44"/>
+      <c r="C16" s="49"/>
+      <c r="D16" s="49"/>
       <c r="G16" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="H16" s="38"/>
-      <c r="I16" s="38"/>
-      <c r="J16" s="38"/>
-      <c r="K16" s="51"/>
+      <c r="H16" s="42"/>
+      <c r="I16" s="42"/>
+      <c r="J16" s="42"/>
+      <c r="K16" s="43"/>
     </row>
     <row r="17" spans="1:11" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="45">
+      <c r="B17" s="50">
         <v>19500</v>
       </c>
-      <c r="C17" s="45"/>
-      <c r="D17" s="45"/>
+      <c r="C17" s="50"/>
+      <c r="D17" s="50"/>
       <c r="G17" s="6" t="s">
         <v>33</v>
       </c>
@@ -1962,11 +1965,11 @@
       <c r="A18" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="46" t="s">
+      <c r="B18" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="46"/>
-      <c r="D18" s="46"/>
+      <c r="C18" s="41"/>
+      <c r="D18" s="41"/>
       <c r="G18" s="6" t="s">
         <v>37</v>
       </c>
@@ -2009,85 +2012,85 @@
       </c>
     </row>
     <row r="20" spans="1:11" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="38" t="s">
+      <c r="A20" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="G20" s="43" t="s">
+      <c r="G20" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="H20" s="43"/>
-      <c r="I20" s="43"/>
-      <c r="J20" s="43"/>
-      <c r="K20" s="43"/>
+      <c r="H20" s="45"/>
+      <c r="I20" s="45"/>
+      <c r="J20" s="45"/>
+      <c r="K20" s="45"/>
     </row>
     <row r="21" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="38"/>
+      <c r="A21" s="42"/>
       <c r="G21" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="H21" s="46">
+      <c r="H21" s="41">
         <v>3.29</v>
       </c>
-      <c r="I21" s="46"/>
-      <c r="J21" s="46"/>
-      <c r="K21" s="46"/>
+      <c r="I21" s="41"/>
+      <c r="J21" s="41"/>
+      <c r="K21" s="41"/>
     </row>
     <row r="22" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="38"/>
+      <c r="A22" s="42"/>
       <c r="G22" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="H22" s="46">
+      <c r="H22" s="41">
         <v>0.03</v>
       </c>
-      <c r="I22" s="46"/>
-      <c r="J22" s="46"/>
-      <c r="K22" s="46"/>
+      <c r="I22" s="41"/>
+      <c r="J22" s="41"/>
+      <c r="K22" s="41"/>
     </row>
     <row r="23" spans="1:11" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="38"/>
+      <c r="A23" s="42"/>
       <c r="G23" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="H23" s="46">
+      <c r="H23" s="41">
         <v>0.01</v>
       </c>
-      <c r="I23" s="46"/>
-      <c r="J23" s="46"/>
-      <c r="K23" s="46"/>
+      <c r="I23" s="41"/>
+      <c r="J23" s="41"/>
+      <c r="K23" s="41"/>
     </row>
     <row r="24" spans="1:11" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="G24" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="H24" s="44">
+      <c r="H24" s="49">
         <v>72</v>
       </c>
-      <c r="I24" s="44"/>
-      <c r="J24" s="44"/>
-      <c r="K24" s="44"/>
+      <c r="I24" s="49"/>
+      <c r="J24" s="49"/>
+      <c r="K24" s="49"/>
     </row>
     <row r="25" spans="1:11" ht="66" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G25" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="H25" s="45">
+      <c r="H25" s="50">
         <v>19500</v>
       </c>
-      <c r="I25" s="45"/>
-      <c r="J25" s="45"/>
-      <c r="K25" s="45"/>
+      <c r="I25" s="50"/>
+      <c r="J25" s="50"/>
+      <c r="K25" s="50"/>
     </row>
     <row r="26" spans="1:11" ht="33.6" x14ac:dyDescent="0.25">
       <c r="G26" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="H26" s="46" t="s">
+      <c r="H26" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="I26" s="46"/>
-      <c r="J26" s="46"/>
-      <c r="K26" s="46"/>
+      <c r="I26" s="41"/>
+      <c r="J26" s="41"/>
+      <c r="K26" s="41"/>
     </row>
     <row r="27" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G27" s="12" t="s">
@@ -2101,7 +2104,7 @@
       <c r="A28" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G28" s="38" t="s">
+      <c r="G28" s="42" t="s">
         <v>45</v>
       </c>
     </row>
@@ -2112,7 +2115,7 @@
       <c r="C29" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="G29" s="38"/>
+      <c r="G29" s="42"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
@@ -2124,7 +2127,7 @@
       <c r="C30" s="1">
         <v>8.6</v>
       </c>
-      <c r="G30" s="38"/>
+      <c r="G30" s="42"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
@@ -2136,7 +2139,7 @@
       <c r="C31" s="1">
         <v>9.5</v>
       </c>
-      <c r="G31" s="38"/>
+      <c r="G31" s="42"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
@@ -2148,7 +2151,7 @@
       <c r="C32" s="1">
         <v>14.1</v>
       </c>
-      <c r="G32" s="38"/>
+      <c r="G32" s="42"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
@@ -2160,7 +2163,7 @@
       <c r="C33" s="1">
         <v>8.1</v>
       </c>
-      <c r="G33" s="38"/>
+      <c r="G33" s="42"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
@@ -2172,7 +2175,7 @@
       <c r="C34" s="1">
         <v>12.3</v>
       </c>
-      <c r="G34" s="38"/>
+      <c r="G34" s="42"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
@@ -2184,7 +2187,7 @@
       <c r="C35" s="1">
         <v>14</v>
       </c>
-      <c r="G35" s="38"/>
+      <c r="G35" s="42"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
@@ -2196,7 +2199,7 @@
       <c r="C36" s="1">
         <v>8</v>
       </c>
-      <c r="G36" s="38"/>
+      <c r="G36" s="42"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
@@ -2208,7 +2211,7 @@
       <c r="C37" s="1">
         <v>4</v>
       </c>
-      <c r="G37" s="38"/>
+      <c r="G37" s="42"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
@@ -2220,7 +2223,7 @@
       <c r="C38" s="1">
         <v>10.1</v>
       </c>
-      <c r="G38" s="38"/>
+      <c r="G38" s="42"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
@@ -2939,36 +2942,36 @@
       </c>
     </row>
     <row r="106" spans="1:34" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A106" s="47" t="s">
+      <c r="A106" s="46" t="s">
         <v>54</v>
       </c>
-      <c r="B106" s="47"/>
-      <c r="D106" s="48" t="s">
+      <c r="B106" s="46"/>
+      <c r="D106" s="47" t="s">
         <v>55</v>
       </c>
-      <c r="E106" s="48"/>
-      <c r="F106" s="48"/>
-      <c r="H106" s="49" t="s">
+      <c r="E106" s="47"/>
+      <c r="F106" s="47"/>
+      <c r="H106" s="48" t="s">
         <v>56</v>
       </c>
-      <c r="I106" s="49"/>
-      <c r="J106" s="49"/>
-      <c r="K106" s="49"/>
-      <c r="L106" s="49"/>
-      <c r="M106" s="49"/>
-      <c r="N106" s="49"/>
-      <c r="O106" s="49"/>
-      <c r="P106" s="49"/>
-      <c r="Q106" s="49"/>
-      <c r="R106" s="49"/>
-      <c r="S106" s="49"/>
-      <c r="V106" s="41" t="s">
+      <c r="I106" s="48"/>
+      <c r="J106" s="48"/>
+      <c r="K106" s="48"/>
+      <c r="L106" s="48"/>
+      <c r="M106" s="48"/>
+      <c r="N106" s="48"/>
+      <c r="O106" s="48"/>
+      <c r="P106" s="48"/>
+      <c r="Q106" s="48"/>
+      <c r="R106" s="48"/>
+      <c r="S106" s="48"/>
+      <c r="V106" s="51" t="s">
         <v>57</v>
       </c>
-      <c r="W106" s="41"/>
-      <c r="X106" s="41"/>
-      <c r="Y106" s="41"/>
-      <c r="Z106" s="41"/>
+      <c r="W106" s="51"/>
+      <c r="X106" s="51"/>
+      <c r="Y106" s="51"/>
+      <c r="Z106" s="51"/>
       <c r="AB106" s="2" t="s">
         <v>58</v>
       </c>
@@ -2992,10 +2995,10 @@
       </c>
     </row>
     <row r="107" spans="1:34" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A107" s="42" t="s">
+      <c r="A107" s="52" t="s">
         <v>65</v>
       </c>
-      <c r="B107" s="42"/>
+      <c r="B107" s="52"/>
       <c r="D107" s="17" t="s">
         <v>66</v>
       </c>
@@ -3738,13 +3741,13 @@
       <c r="T116" s="1">
         <v>0.118312327125455</v>
       </c>
-      <c r="V116" s="43" t="s">
+      <c r="V116" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="W116" s="43"/>
-      <c r="X116" s="43"/>
-      <c r="Y116" s="43"/>
-      <c r="Z116" s="43"/>
+      <c r="W116" s="45"/>
+      <c r="X116" s="45"/>
+      <c r="Y116" s="45"/>
+      <c r="Z116" s="45"/>
       <c r="AB116" s="1">
         <v>72</v>
       </c>
@@ -3816,14 +3819,14 @@
       <c r="V117" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="W117" s="38">
+      <c r="W117" s="42">
         <v>3.29</v>
       </c>
-      <c r="X117" s="38"/>
-      <c r="Y117" s="38">
+      <c r="X117" s="42"/>
+      <c r="Y117" s="42">
         <v>3.29</v>
       </c>
-      <c r="Z117" s="38"/>
+      <c r="Z117" s="42"/>
       <c r="AB117" s="1">
         <v>71</v>
       </c>
@@ -3895,14 +3898,14 @@
       <c r="V118" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="W118" s="38" t="s">
+      <c r="W118" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="X118" s="38"/>
-      <c r="Y118" s="38" t="s">
+      <c r="X118" s="42"/>
+      <c r="Y118" s="42" t="s">
         <v>126</v>
       </c>
-      <c r="Z118" s="38"/>
+      <c r="Z118" s="42"/>
       <c r="AB118" s="1">
         <v>70</v>
       </c>
@@ -3974,14 +3977,14 @@
       <c r="V119" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="W119" s="38">
+      <c r="W119" s="42">
         <v>0.08</v>
       </c>
-      <c r="X119" s="38"/>
-      <c r="Y119" s="38">
+      <c r="X119" s="42"/>
+      <c r="Y119" s="42">
         <v>0.01</v>
       </c>
-      <c r="Z119" s="38"/>
+      <c r="Z119" s="42"/>
       <c r="AB119" s="1">
         <v>64</v>
       </c>
@@ -4051,14 +4054,14 @@
       <c r="V120" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="W120" s="39" t="s">
+      <c r="W120" s="56" t="s">
         <v>130</v>
       </c>
-      <c r="X120" s="39"/>
-      <c r="Y120" s="39" t="s">
+      <c r="X120" s="56"/>
+      <c r="Y120" s="56" t="s">
         <v>130</v>
       </c>
-      <c r="Z120" s="39"/>
+      <c r="Z120" s="56"/>
       <c r="AB120" s="1">
         <v>69</v>
       </c>
@@ -4130,14 +4133,14 @@
       <c r="V121" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="W121" s="40">
+      <c r="W121" s="57">
         <v>19500</v>
       </c>
-      <c r="X121" s="40"/>
-      <c r="Y121" s="40">
+      <c r="X121" s="57"/>
+      <c r="Y121" s="57">
         <v>19500</v>
       </c>
-      <c r="Z121" s="40"/>
+      <c r="Z121" s="57"/>
       <c r="AB121" s="1">
         <v>68</v>
       </c>
@@ -4209,14 +4212,14 @@
       <c r="V122" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="W122" s="35" t="s">
+      <c r="W122" s="53" t="s">
         <v>36</v>
       </c>
-      <c r="X122" s="35"/>
-      <c r="Y122" s="35" t="s">
+      <c r="X122" s="53"/>
+      <c r="Y122" s="53" t="s">
         <v>43</v>
       </c>
-      <c r="Z122" s="35"/>
+      <c r="Z122" s="53"/>
     </row>
     <row r="123" spans="1:34" ht="42" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A123" s="25" t="s">
@@ -4262,13 +4265,13 @@
       <c r="T123" s="1">
         <v>4.6341574791248501E-2</v>
       </c>
-      <c r="V123" s="36" t="s">
+      <c r="V123" s="54" t="s">
         <v>136</v>
       </c>
-      <c r="W123" s="36"/>
-      <c r="X123" s="36"/>
-      <c r="Y123" s="36"/>
-      <c r="Z123" s="36"/>
+      <c r="W123" s="54"/>
+      <c r="X123" s="54"/>
+      <c r="Y123" s="54"/>
+      <c r="Z123" s="54"/>
     </row>
     <row r="124" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="26" t="s">
@@ -4530,10 +4533,10 @@
       <c r="AC128" s="19"/>
     </row>
     <row r="129" spans="1:29" ht="16.8" x14ac:dyDescent="0.25">
-      <c r="A129" s="37" t="s">
+      <c r="A129" s="55" t="s">
         <v>150</v>
       </c>
-      <c r="B129" s="37"/>
+      <c r="B129" s="55"/>
       <c r="H129" s="20" t="s">
         <v>76</v>
       </c>
@@ -6687,16 +6690,26 @@
     </row>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="K15:K16"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="H9:K9"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="V123:Z123"/>
+    <mergeCell ref="A129:B129"/>
+    <mergeCell ref="W119:X119"/>
+    <mergeCell ref="Y119:Z119"/>
+    <mergeCell ref="W120:X120"/>
+    <mergeCell ref="Y120:Z120"/>
+    <mergeCell ref="W121:X121"/>
+    <mergeCell ref="Y121:Z121"/>
+    <mergeCell ref="A107:B107"/>
+    <mergeCell ref="V116:Z116"/>
+    <mergeCell ref="W117:X117"/>
+    <mergeCell ref="Y117:Z117"/>
+    <mergeCell ref="W122:X122"/>
+    <mergeCell ref="Y122:Z122"/>
+    <mergeCell ref="W118:X118"/>
+    <mergeCell ref="Y118:Z118"/>
+    <mergeCell ref="H24:K24"/>
+    <mergeCell ref="H25:K25"/>
+    <mergeCell ref="H26:K26"/>
+    <mergeCell ref="V106:Z106"/>
     <mergeCell ref="G28:G38"/>
     <mergeCell ref="A106:B106"/>
     <mergeCell ref="D106:F106"/>
@@ -6709,26 +6722,16 @@
     <mergeCell ref="H21:K21"/>
     <mergeCell ref="H22:K22"/>
     <mergeCell ref="H23:K23"/>
-    <mergeCell ref="W118:X118"/>
-    <mergeCell ref="Y118:Z118"/>
-    <mergeCell ref="H24:K24"/>
-    <mergeCell ref="H25:K25"/>
-    <mergeCell ref="H26:K26"/>
-    <mergeCell ref="V106:Z106"/>
-    <mergeCell ref="A107:B107"/>
-    <mergeCell ref="V116:Z116"/>
-    <mergeCell ref="W117:X117"/>
-    <mergeCell ref="Y117:Z117"/>
-    <mergeCell ref="W122:X122"/>
-    <mergeCell ref="Y122:Z122"/>
-    <mergeCell ref="V123:Z123"/>
-    <mergeCell ref="A129:B129"/>
-    <mergeCell ref="W119:X119"/>
-    <mergeCell ref="Y119:Z119"/>
-    <mergeCell ref="W120:X120"/>
-    <mergeCell ref="Y120:Z120"/>
-    <mergeCell ref="W121:X121"/>
-    <mergeCell ref="Y121:Z121"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="H9:K9"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="K15:K16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6771,31 +6774,31 @@
     </row>
     <row r="3" spans="1:21" ht="28.2" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="50"/>
-      <c r="D3" s="50"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
       <c r="F3" s="3"/>
-      <c r="G3" s="50" t="s">
+      <c r="G3" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="50"/>
-      <c r="I3" s="50"/>
-      <c r="J3" s="50"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="44"/>
       <c r="L3" s="3"/>
-      <c r="M3" s="50" t="s">
+      <c r="M3" s="44" t="s">
         <v>164</v>
       </c>
-      <c r="N3" s="50"/>
-      <c r="O3" s="50"/>
+      <c r="N3" s="44"/>
+      <c r="O3" s="44"/>
       <c r="Q3" s="3"/>
-      <c r="R3" s="50" t="s">
+      <c r="R3" s="44" t="s">
         <v>164</v>
       </c>
-      <c r="S3" s="50"/>
-      <c r="T3" s="50"/>
-      <c r="U3" s="50"/>
+      <c r="S3" s="44"/>
+      <c r="T3" s="44"/>
+      <c r="U3" s="44"/>
     </row>
     <row r="4" spans="1:21" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
@@ -6910,12 +6913,12 @@
       </c>
     </row>
     <row r="6" spans="1:21" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="43"/>
-      <c r="C6" s="43"/>
-      <c r="D6" s="43"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
       <c r="F6" s="6" t="s">
         <v>19</v>
       </c>
@@ -6931,12 +6934,12 @@
       <c r="J6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="L6" s="43" t="s">
+      <c r="L6" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="M6" s="43"/>
-      <c r="N6" s="43"/>
-      <c r="O6" s="43"/>
+      <c r="M6" s="45"/>
+      <c r="N6" s="45"/>
+      <c r="O6" s="45"/>
       <c r="Q6" s="6" t="s">
         <v>19</v>
       </c>
@@ -6957,11 +6960,11 @@
       <c r="A7" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="46">
+      <c r="B7" s="41">
         <v>3.29</v>
       </c>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="41"/>
       <c r="F7" s="6" t="s">
         <v>172</v>
       </c>
@@ -6980,11 +6983,11 @@
       <c r="L7" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="M7" s="46">
+      <c r="M7" s="41">
         <v>0.59</v>
       </c>
-      <c r="N7" s="46"/>
-      <c r="O7" s="46"/>
+      <c r="N7" s="41"/>
+      <c r="O7" s="41"/>
       <c r="Q7" s="6" t="s">
         <v>172</v>
       </c>
@@ -7005,11 +7008,11 @@
       <c r="A8" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="46">
+      <c r="B8" s="41">
         <v>0.9</v>
       </c>
-      <c r="C8" s="46"/>
-      <c r="D8" s="46"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="41"/>
       <c r="F8" s="6" t="s">
         <v>175</v>
       </c>
@@ -7028,11 +7031,11 @@
       <c r="L8" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="M8" s="46">
+      <c r="M8" s="41">
         <v>0.01</v>
       </c>
-      <c r="N8" s="46"/>
-      <c r="O8" s="46"/>
+      <c r="N8" s="41"/>
+      <c r="O8" s="41"/>
       <c r="Q8" s="6" t="s">
         <v>175</v>
       </c>
@@ -7053,11 +7056,11 @@
       <c r="A9" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="46">
+      <c r="B9" s="41">
         <v>0.21</v>
       </c>
-      <c r="C9" s="46"/>
-      <c r="D9" s="46"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="41"/>
       <c r="F9" s="6" t="s">
         <v>178</v>
       </c>
@@ -7076,11 +7079,11 @@
       <c r="L9" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="M9" s="46">
+      <c r="M9" s="41">
         <v>0.02</v>
       </c>
-      <c r="N9" s="46"/>
-      <c r="O9" s="46"/>
+      <c r="N9" s="41"/>
+      <c r="O9" s="41"/>
       <c r="Q9" s="6" t="s">
         <v>178</v>
       </c>
@@ -7101,11 +7104,11 @@
       <c r="A10" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="44">
+      <c r="B10" s="49">
         <v>108</v>
       </c>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
       <c r="F10" s="6" t="s">
         <v>181</v>
       </c>
@@ -7124,11 +7127,11 @@
       <c r="L10" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="M10" s="44">
+      <c r="M10" s="49">
         <v>108</v>
       </c>
-      <c r="N10" s="44"/>
-      <c r="O10" s="44"/>
+      <c r="N10" s="49"/>
+      <c r="O10" s="49"/>
       <c r="Q10" s="6" t="s">
         <v>181</v>
       </c>
@@ -7149,11 +7152,11 @@
       <c r="A11" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="45">
+      <c r="B11" s="50">
         <v>29653</v>
       </c>
-      <c r="C11" s="45"/>
-      <c r="D11" s="45"/>
+      <c r="C11" s="50"/>
+      <c r="D11" s="50"/>
       <c r="F11" s="6" t="s">
         <v>184</v>
       </c>
@@ -7172,11 +7175,11 @@
       <c r="L11" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="M11" s="45">
+      <c r="M11" s="50">
         <v>29653</v>
       </c>
-      <c r="N11" s="45"/>
-      <c r="O11" s="45"/>
+      <c r="N11" s="50"/>
+      <c r="O11" s="50"/>
       <c r="Q11" s="6" t="s">
         <v>184</v>
       </c>
@@ -7197,11 +7200,11 @@
       <c r="A12" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="46" t="s">
+      <c r="B12" s="41" t="s">
         <v>187</v>
       </c>
-      <c r="C12" s="46"/>
-      <c r="D12" s="46"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
       <c r="F12" s="6" t="s">
         <v>188</v>
       </c>
@@ -7220,11 +7223,11 @@
       <c r="L12" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="M12" s="46" t="s">
+      <c r="M12" s="41" t="s">
         <v>190</v>
       </c>
-      <c r="N12" s="46"/>
-      <c r="O12" s="46"/>
+      <c r="N12" s="41"/>
+      <c r="O12" s="41"/>
       <c r="Q12" s="6" t="s">
         <v>188</v>
       </c>
@@ -7245,7 +7248,7 @@
       <c r="A13" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="52">
+      <c r="B13" s="35">
         <v>21.405159999999999</v>
       </c>
       <c r="F13" s="6" t="s">
@@ -7266,7 +7269,7 @@
       <c r="L13" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="M13" s="52">
+      <c r="M13" s="35">
         <v>2.307426</v>
       </c>
       <c r="Q13" s="6" t="s">
@@ -7350,13 +7353,13 @@
       </c>
     </row>
     <row r="16" spans="1:21" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F16" s="43" t="s">
+      <c r="F16" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="G16" s="43"/>
-      <c r="H16" s="43"/>
-      <c r="I16" s="43"/>
-      <c r="J16" s="43"/>
+      <c r="G16" s="45"/>
+      <c r="H16" s="45"/>
+      <c r="I16" s="45"/>
+      <c r="J16" s="45"/>
       <c r="Q16" s="9" t="s">
         <v>18</v>
       </c>
@@ -7369,12 +7372,12 @@
       <c r="F17" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G17" s="46">
+      <c r="G17" s="41">
         <v>3.29</v>
       </c>
-      <c r="H17" s="46"/>
-      <c r="I17" s="46"/>
-      <c r="J17" s="46"/>
+      <c r="H17" s="41"/>
+      <c r="I17" s="41"/>
+      <c r="J17" s="41"/>
       <c r="Q17" s="6" t="s">
         <v>21</v>
       </c>
@@ -7383,12 +7386,12 @@
       <c r="F18" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="G18" s="46">
+      <c r="G18" s="41">
         <v>0.02</v>
       </c>
-      <c r="H18" s="46"/>
-      <c r="I18" s="46"/>
-      <c r="J18" s="46"/>
+      <c r="H18" s="41"/>
+      <c r="I18" s="41"/>
+      <c r="J18" s="41"/>
       <c r="Q18" s="6" t="s">
         <v>24</v>
       </c>
@@ -7403,12 +7406,12 @@
       <c r="F19" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G19" s="46">
+      <c r="G19" s="41">
         <v>0.01</v>
       </c>
-      <c r="H19" s="46"/>
-      <c r="I19" s="46"/>
-      <c r="J19" s="46"/>
+      <c r="H19" s="41"/>
+      <c r="I19" s="41"/>
+      <c r="J19" s="41"/>
       <c r="Q19" s="6" t="s">
         <v>30</v>
       </c>
@@ -7423,12 +7426,12 @@
       <c r="F20" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="G20" s="44">
+      <c r="G20" s="49">
         <v>108</v>
       </c>
-      <c r="H20" s="44"/>
-      <c r="I20" s="44"/>
-      <c r="J20" s="44"/>
+      <c r="H20" s="49"/>
+      <c r="I20" s="49"/>
+      <c r="J20" s="49"/>
       <c r="Q20" s="11" t="s">
         <v>32</v>
       </c>
@@ -7443,16 +7446,16 @@
       <c r="F21" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="G21" s="45">
+      <c r="G21" s="50">
         <v>29653</v>
       </c>
-      <c r="H21" s="45"/>
-      <c r="I21" s="45"/>
-      <c r="J21" s="45"/>
+      <c r="H21" s="50"/>
+      <c r="I21" s="50"/>
+      <c r="J21" s="50"/>
       <c r="Q21" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="R21" s="53">
+      <c r="R21" s="36">
         <v>3.6478820000000001E-8</v>
       </c>
     </row>
@@ -7460,23 +7463,41 @@
       <c r="F22" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="G22" s="46" t="s">
+      <c r="G22" s="41" t="s">
         <v>199</v>
       </c>
-      <c r="H22" s="46"/>
-      <c r="I22" s="46"/>
-      <c r="J22" s="46"/>
+      <c r="H22" s="41"/>
+      <c r="I22" s="41"/>
+      <c r="J22" s="41"/>
     </row>
     <row r="23" spans="6:21" x14ac:dyDescent="0.3">
       <c r="F23" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G23" s="52">
+      <c r="G23" s="35">
         <v>0.6992389</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="M3:O3"/>
+    <mergeCell ref="R3:U3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="L6:O6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="M7:O7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="M8:O8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="M9:O9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="M10:O10"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="M12:O12"/>
     <mergeCell ref="G22:J22"/>
     <mergeCell ref="F16:J16"/>
     <mergeCell ref="G17:J17"/>
@@ -7484,24 +7505,6 @@
     <mergeCell ref="G19:J19"/>
     <mergeCell ref="G20:J20"/>
     <mergeCell ref="G21:J21"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="M10:O10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="M12:O12"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="M7:O7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="M8:O8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="M9:O9"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="G3:J3"/>
-    <mergeCell ref="M3:O3"/>
-    <mergeCell ref="R3:U3"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="L6:O6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7529,36 +7532,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="37" t="s">
         <v>159</v>
       </c>
-      <c r="X1" s="54" t="s">
+      <c r="X1" s="37" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:44" x14ac:dyDescent="0.3">
-      <c r="A2" s="54" t="s">
+      <c r="A2" s="37" t="s">
         <v>200</v>
       </c>
-      <c r="F2" s="54" t="s">
+      <c r="F2" s="37" t="s">
         <v>201</v>
       </c>
-      <c r="L2" s="54" t="s">
+      <c r="L2" s="37" t="s">
         <v>161</v>
       </c>
-      <c r="Q2" s="54" t="s">
+      <c r="Q2" s="37" t="s">
         <v>162</v>
       </c>
-      <c r="X2" s="54" t="s">
+      <c r="X2" s="37" t="s">
         <v>202</v>
       </c>
-      <c r="AC2" s="54" t="s">
+      <c r="AC2" s="37" t="s">
         <v>203</v>
       </c>
-      <c r="AI2" s="54" t="s">
+      <c r="AI2" s="37" t="s">
         <v>163</v>
       </c>
-      <c r="AN2" s="54" t="s">
+      <c r="AN2" s="37" t="s">
         <v>204</v>
       </c>
     </row>
@@ -7578,57 +7581,57 @@
     </row>
     <row r="4" spans="1:44" ht="28.2" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
-      <c r="B4" s="50" t="s">
+      <c r="B4" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="50"/>
-      <c r="D4" s="50"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
       <c r="F4" s="3"/>
-      <c r="G4" s="50" t="s">
+      <c r="G4" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="50"/>
-      <c r="I4" s="50"/>
-      <c r="J4" s="50"/>
-      <c r="L4" s="50" t="s">
+      <c r="H4" s="44"/>
+      <c r="I4" s="44"/>
+      <c r="J4" s="44"/>
+      <c r="L4" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="M4" s="50"/>
-      <c r="N4" s="50"/>
-      <c r="O4" s="50"/>
+      <c r="M4" s="44"/>
+      <c r="N4" s="44"/>
+      <c r="O4" s="44"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="50" t="s">
+      <c r="R4" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="S4" s="50"/>
-      <c r="T4" s="50"/>
-      <c r="U4" s="50"/>
-      <c r="X4" s="50" t="s">
+      <c r="S4" s="44"/>
+      <c r="T4" s="44"/>
+      <c r="U4" s="44"/>
+      <c r="X4" s="44" t="s">
         <v>164</v>
       </c>
-      <c r="Y4" s="50"/>
-      <c r="Z4" s="50"/>
-      <c r="AA4" s="50"/>
-      <c r="AC4" s="50" t="s">
+      <c r="Y4" s="44"/>
+      <c r="Z4" s="44"/>
+      <c r="AA4" s="44"/>
+      <c r="AC4" s="44" t="s">
         <v>164</v>
       </c>
-      <c r="AD4" s="50"/>
-      <c r="AE4" s="50"/>
-      <c r="AF4" s="50"/>
-      <c r="AG4" s="50"/>
-      <c r="AI4" s="50" t="s">
+      <c r="AD4" s="44"/>
+      <c r="AE4" s="44"/>
+      <c r="AF4" s="44"/>
+      <c r="AG4" s="44"/>
+      <c r="AI4" s="44" t="s">
         <v>164</v>
       </c>
-      <c r="AJ4" s="50"/>
-      <c r="AK4" s="50"/>
-      <c r="AL4" s="50"/>
-      <c r="AN4" s="50" t="s">
+      <c r="AJ4" s="44"/>
+      <c r="AK4" s="44"/>
+      <c r="AL4" s="44"/>
+      <c r="AN4" s="44" t="s">
         <v>164</v>
       </c>
-      <c r="AO4" s="50"/>
-      <c r="AP4" s="50"/>
-      <c r="AQ4" s="50"/>
-      <c r="AR4" s="50"/>
+      <c r="AO4" s="44"/>
+      <c r="AP4" s="44"/>
+      <c r="AQ4" s="44"/>
+      <c r="AR4" s="44"/>
     </row>
     <row r="5" spans="1:44" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
@@ -7851,12 +7854,12 @@
       </c>
     </row>
     <row r="7" spans="1:44" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="43"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="45"/>
+      <c r="D7" s="45"/>
       <c r="F7" s="6" t="s">
         <v>19</v>
       </c>
@@ -7872,12 +7875,12 @@
       <c r="J7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="L7" s="43" t="s">
+      <c r="L7" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="M7" s="43"/>
-      <c r="N7" s="43"/>
-      <c r="O7" s="43"/>
+      <c r="M7" s="45"/>
+      <c r="N7" s="45"/>
+      <c r="O7" s="45"/>
       <c r="Q7" s="6" t="s">
         <v>19</v>
       </c>
@@ -7893,12 +7896,12 @@
       <c r="U7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="X7" s="43" t="s">
+      <c r="X7" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="Y7" s="43"/>
-      <c r="Z7" s="43"/>
-      <c r="AA7" s="43"/>
+      <c r="Y7" s="45"/>
+      <c r="Z7" s="45"/>
+      <c r="AA7" s="45"/>
       <c r="AC7" s="6" t="s">
         <v>19</v>
       </c>
@@ -7914,12 +7917,12 @@
       <c r="AG7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="AI7" s="43" t="s">
+      <c r="AI7" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="AJ7" s="43"/>
-      <c r="AK7" s="43"/>
-      <c r="AL7" s="43"/>
+      <c r="AJ7" s="45"/>
+      <c r="AK7" s="45"/>
+      <c r="AL7" s="45"/>
       <c r="AN7" s="6" t="s">
         <v>19</v>
       </c>
@@ -7940,11 +7943,11 @@
       <c r="A8" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="46">
+      <c r="B8" s="41">
         <v>3.29</v>
       </c>
-      <c r="C8" s="46"/>
-      <c r="D8" s="46"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="41"/>
       <c r="F8" s="6" t="s">
         <v>22</v>
       </c>
@@ -7963,11 +7966,11 @@
       <c r="L8" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="M8" s="46">
+      <c r="M8" s="41">
         <v>3.29</v>
       </c>
-      <c r="N8" s="46"/>
-      <c r="O8" s="46"/>
+      <c r="N8" s="41"/>
+      <c r="O8" s="41"/>
       <c r="Q8" s="6" t="s">
         <v>22</v>
       </c>
@@ -7986,11 +7989,11 @@
       <c r="X8" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="Y8" s="46">
+      <c r="Y8" s="41">
         <v>2.12</v>
       </c>
-      <c r="Z8" s="46"/>
-      <c r="AA8" s="46"/>
+      <c r="Z8" s="41"/>
+      <c r="AA8" s="41"/>
       <c r="AC8" s="6" t="s">
         <v>22</v>
       </c>
@@ -8009,11 +8012,11 @@
       <c r="AI8" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="AJ8" s="46">
+      <c r="AJ8" s="41">
         <v>2.11</v>
       </c>
-      <c r="AK8" s="46"/>
-      <c r="AL8" s="46"/>
+      <c r="AK8" s="41"/>
+      <c r="AL8" s="41"/>
       <c r="AN8" s="6" t="s">
         <v>22</v>
       </c>
@@ -8034,11 +8037,11 @@
       <c r="A9" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="46">
+      <c r="B9" s="41">
         <v>0.24</v>
       </c>
-      <c r="C9" s="46"/>
-      <c r="D9" s="46"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="41"/>
       <c r="F9" s="6" t="s">
         <v>25</v>
       </c>
@@ -8057,11 +8060,11 @@
       <c r="L9" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="M9" s="46">
+      <c r="M9" s="41">
         <v>0.26</v>
       </c>
-      <c r="N9" s="46"/>
-      <c r="O9" s="46"/>
+      <c r="N9" s="41"/>
+      <c r="O9" s="41"/>
       <c r="Q9" s="6" t="s">
         <v>25</v>
       </c>
@@ -8080,11 +8083,11 @@
       <c r="X9" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="Y9" s="46">
+      <c r="Y9" s="41">
         <v>0.17</v>
       </c>
-      <c r="Z9" s="46"/>
-      <c r="AA9" s="46"/>
+      <c r="Z9" s="41"/>
+      <c r="AA9" s="41"/>
       <c r="AC9" s="6" t="s">
         <v>25</v>
       </c>
@@ -8103,11 +8106,11 @@
       <c r="AI9" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="AJ9" s="46">
+      <c r="AJ9" s="41">
         <v>0.18</v>
       </c>
-      <c r="AK9" s="46"/>
-      <c r="AL9" s="46"/>
+      <c r="AK9" s="41"/>
+      <c r="AL9" s="41"/>
       <c r="AN9" s="6" t="s">
         <v>25</v>
       </c>
@@ -8128,11 +8131,11 @@
       <c r="A10" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="46">
+      <c r="B10" s="41">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="C10" s="46"/>
-      <c r="D10" s="46"/>
+      <c r="C10" s="41"/>
+      <c r="D10" s="41"/>
       <c r="F10" s="6" t="s">
         <v>224</v>
       </c>
@@ -8151,11 +8154,11 @@
       <c r="L10" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="M10" s="46">
+      <c r="M10" s="41">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N10" s="46"/>
-      <c r="O10" s="46"/>
+      <c r="N10" s="41"/>
+      <c r="O10" s="41"/>
       <c r="Q10" s="6" t="s">
         <v>178</v>
       </c>
@@ -8174,11 +8177,11 @@
       <c r="X10" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="Y10" s="46">
+      <c r="Y10" s="41">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="Z10" s="46"/>
-      <c r="AA10" s="46"/>
+      <c r="Z10" s="41"/>
+      <c r="AA10" s="41"/>
       <c r="AC10" s="6" t="s">
         <v>224</v>
       </c>
@@ -8197,11 +8200,11 @@
       <c r="AI10" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="AJ10" s="46">
+      <c r="AJ10" s="41">
         <v>0.08</v>
       </c>
-      <c r="AK10" s="46"/>
-      <c r="AL10" s="46"/>
+      <c r="AK10" s="41"/>
+      <c r="AL10" s="41"/>
       <c r="AN10" s="6" t="s">
         <v>178</v>
       </c>
@@ -8222,11 +8225,11 @@
       <c r="A11" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="44">
+      <c r="B11" s="49">
         <v>54</v>
       </c>
-      <c r="C11" s="44"/>
-      <c r="D11" s="44"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49"/>
       <c r="F11" s="6" t="s">
         <v>229</v>
       </c>
@@ -8245,11 +8248,11 @@
       <c r="L11" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="M11" s="44">
+      <c r="M11" s="49">
         <v>108</v>
       </c>
-      <c r="N11" s="44"/>
-      <c r="O11" s="44"/>
+      <c r="N11" s="49"/>
+      <c r="O11" s="49"/>
       <c r="Q11" s="6" t="s">
         <v>181</v>
       </c>
@@ -8268,11 +8271,11 @@
       <c r="X11" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="Y11" s="44">
+      <c r="Y11" s="49">
         <v>54</v>
       </c>
-      <c r="Z11" s="44"/>
-      <c r="AA11" s="44"/>
+      <c r="Z11" s="49"/>
+      <c r="AA11" s="49"/>
       <c r="AC11" s="6" t="s">
         <v>229</v>
       </c>
@@ -8291,11 +8294,11 @@
       <c r="AI11" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="AJ11" s="44">
+      <c r="AJ11" s="49">
         <v>108</v>
       </c>
-      <c r="AK11" s="44"/>
-      <c r="AL11" s="44"/>
+      <c r="AK11" s="49"/>
+      <c r="AL11" s="49"/>
       <c r="AN11" s="6" t="s">
         <v>181</v>
       </c>
@@ -8316,11 +8319,11 @@
       <c r="A12" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="45">
+      <c r="B12" s="50">
         <v>19500</v>
       </c>
-      <c r="C12" s="45"/>
-      <c r="D12" s="45"/>
+      <c r="C12" s="50"/>
+      <c r="D12" s="50"/>
       <c r="F12" s="6" t="s">
         <v>33</v>
       </c>
@@ -8339,11 +8342,11 @@
       <c r="L12" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="M12" s="45">
+      <c r="M12" s="50">
         <v>19500</v>
       </c>
-      <c r="N12" s="45"/>
-      <c r="O12" s="45"/>
+      <c r="N12" s="50"/>
+      <c r="O12" s="50"/>
       <c r="Q12" s="6" t="s">
         <v>184</v>
       </c>
@@ -8362,11 +8365,11 @@
       <c r="X12" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="Y12" s="45">
+      <c r="Y12" s="50">
         <v>19500</v>
       </c>
-      <c r="Z12" s="45"/>
-      <c r="AA12" s="45"/>
+      <c r="Z12" s="50"/>
+      <c r="AA12" s="50"/>
       <c r="AC12" s="6" t="s">
         <v>33</v>
       </c>
@@ -8385,11 +8388,11 @@
       <c r="AI12" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="AJ12" s="45">
+      <c r="AJ12" s="50">
         <v>19500</v>
       </c>
-      <c r="AK12" s="45"/>
-      <c r="AL12" s="45"/>
+      <c r="AK12" s="50"/>
+      <c r="AL12" s="50"/>
       <c r="AN12" s="6" t="s">
         <v>184</v>
       </c>
@@ -8410,11 +8413,11 @@
       <c r="A13" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="46" t="s">
+      <c r="B13" s="41" t="s">
         <v>237</v>
       </c>
-      <c r="C13" s="46"/>
-      <c r="D13" s="46"/>
+      <c r="C13" s="41"/>
+      <c r="D13" s="41"/>
       <c r="F13" s="6" t="s">
         <v>37</v>
       </c>
@@ -8433,11 +8436,11 @@
       <c r="L13" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="M13" s="46" t="s">
+      <c r="M13" s="41" t="s">
         <v>239</v>
       </c>
-      <c r="N13" s="46"/>
-      <c r="O13" s="46"/>
+      <c r="N13" s="41"/>
+      <c r="O13" s="41"/>
       <c r="Q13" s="6" t="s">
         <v>188</v>
       </c>
@@ -8456,11 +8459,11 @@
       <c r="X13" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="Y13" s="46" t="s">
+      <c r="Y13" s="41" t="s">
         <v>239</v>
       </c>
-      <c r="Z13" s="46"/>
-      <c r="AA13" s="46"/>
+      <c r="Z13" s="41"/>
+      <c r="AA13" s="41"/>
       <c r="AC13" s="6" t="s">
         <v>37</v>
       </c>
@@ -8479,11 +8482,11 @@
       <c r="AI13" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="AJ13" s="46" t="s">
+      <c r="AJ13" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="AK13" s="46"/>
-      <c r="AL13" s="46"/>
+      <c r="AK13" s="41"/>
+      <c r="AL13" s="41"/>
       <c r="AN13" s="6" t="s">
         <v>188</v>
       </c>
@@ -8507,15 +8510,15 @@
       <c r="B14" s="13">
         <v>6.678481E-2</v>
       </c>
-      <c r="C14" s="55"/>
-      <c r="D14" s="55"/>
-      <c r="F14" s="43" t="s">
+      <c r="C14" s="38"/>
+      <c r="D14" s="38"/>
+      <c r="F14" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="G14" s="43"/>
-      <c r="H14" s="43"/>
-      <c r="I14" s="43"/>
-      <c r="J14" s="43"/>
+      <c r="G14" s="45"/>
+      <c r="H14" s="45"/>
+      <c r="I14" s="45"/>
+      <c r="J14" s="45"/>
       <c r="L14" s="12" t="s">
         <v>39</v>
       </c>
@@ -8545,17 +8548,17 @@
       </c>
       <c r="Z14" s="14"/>
       <c r="AA14" s="14"/>
-      <c r="AC14" s="43" t="s">
+      <c r="AC14" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="AD14" s="43"/>
-      <c r="AE14" s="43"/>
-      <c r="AF14" s="43"/>
-      <c r="AG14" s="43"/>
+      <c r="AD14" s="45"/>
+      <c r="AE14" s="45"/>
+      <c r="AF14" s="45"/>
+      <c r="AG14" s="45"/>
       <c r="AI14" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="AJ14" s="56">
+      <c r="AJ14" s="39">
         <v>7.5683070000000005E-2</v>
       </c>
       <c r="AN14" s="6" t="s">
@@ -8575,18 +8578,18 @@
       </c>
     </row>
     <row r="15" spans="1:44" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="38" t="s">
+      <c r="A15" s="42" t="s">
         <v>246</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G15" s="46">
+      <c r="G15" s="41">
         <v>3.29</v>
       </c>
-      <c r="H15" s="46"/>
-      <c r="I15" s="46"/>
-      <c r="J15" s="46"/>
+      <c r="H15" s="41"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="41"/>
       <c r="Q15" s="6" t="s">
         <v>33</v>
       </c>
@@ -8605,12 +8608,12 @@
       <c r="AC15" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="AD15" s="46">
+      <c r="AD15" s="41">
         <v>2.12</v>
       </c>
-      <c r="AE15" s="46"/>
-      <c r="AF15" s="46"/>
-      <c r="AG15" s="46"/>
+      <c r="AE15" s="41"/>
+      <c r="AF15" s="41"/>
+      <c r="AG15" s="41"/>
       <c r="AN15" s="6" t="s">
         <v>33</v>
       </c>
@@ -8628,16 +8631,16 @@
       </c>
     </row>
     <row r="16" spans="1:44" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="38"/>
+      <c r="A16" s="42"/>
       <c r="F16" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="G16" s="46">
+      <c r="G16" s="41">
         <v>0.01</v>
       </c>
-      <c r="H16" s="46"/>
-      <c r="I16" s="46"/>
-      <c r="J16" s="46"/>
+      <c r="H16" s="41"/>
+      <c r="I16" s="41"/>
+      <c r="J16" s="41"/>
       <c r="Q16" s="6" t="s">
         <v>37</v>
       </c>
@@ -8656,12 +8659,12 @@
       <c r="AC16" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="AD16" s="46">
+      <c r="AD16" s="41">
         <v>0</v>
       </c>
-      <c r="AE16" s="46"/>
-      <c r="AF16" s="46"/>
-      <c r="AG16" s="46"/>
+      <c r="AE16" s="41"/>
+      <c r="AF16" s="41"/>
+      <c r="AG16" s="41"/>
       <c r="AN16" s="6" t="s">
         <v>37</v>
       </c>
@@ -8679,154 +8682,154 @@
       </c>
     </row>
     <row r="17" spans="1:44" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="38"/>
+      <c r="A17" s="42"/>
       <c r="F17" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G17" s="46">
+      <c r="G17" s="41">
         <v>0</v>
       </c>
-      <c r="H17" s="46"/>
-      <c r="I17" s="46"/>
-      <c r="J17" s="46"/>
-      <c r="Q17" s="43" t="s">
+      <c r="H17" s="41"/>
+      <c r="I17" s="41"/>
+      <c r="J17" s="41"/>
+      <c r="Q17" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="R17" s="43"/>
-      <c r="S17" s="43"/>
-      <c r="T17" s="43"/>
-      <c r="U17" s="43"/>
+      <c r="R17" s="45"/>
+      <c r="S17" s="45"/>
+      <c r="T17" s="45"/>
+      <c r="U17" s="45"/>
       <c r="AC17" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="AD17" s="46">
+      <c r="AD17" s="41">
         <v>0</v>
       </c>
-      <c r="AE17" s="46"/>
-      <c r="AF17" s="46"/>
-      <c r="AG17" s="46"/>
-      <c r="AN17" s="43" t="s">
+      <c r="AE17" s="41"/>
+      <c r="AF17" s="41"/>
+      <c r="AG17" s="41"/>
+      <c r="AN17" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="AO17" s="43"/>
-      <c r="AP17" s="43"/>
-      <c r="AQ17" s="43"/>
-      <c r="AR17" s="43"/>
+      <c r="AO17" s="45"/>
+      <c r="AP17" s="45"/>
+      <c r="AQ17" s="45"/>
+      <c r="AR17" s="45"/>
     </row>
     <row r="18" spans="1:44" ht="28.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="38"/>
+      <c r="A18" s="42"/>
       <c r="F18" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="G18" s="44">
+      <c r="G18" s="49">
         <v>54</v>
       </c>
-      <c r="H18" s="44"/>
-      <c r="I18" s="44"/>
-      <c r="J18" s="44"/>
+      <c r="H18" s="49"/>
+      <c r="I18" s="49"/>
+      <c r="J18" s="49"/>
       <c r="Q18" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="R18" s="46">
+      <c r="R18" s="41">
         <v>3.29</v>
       </c>
-      <c r="S18" s="46"/>
-      <c r="T18" s="46"/>
-      <c r="U18" s="46"/>
+      <c r="S18" s="41"/>
+      <c r="T18" s="41"/>
+      <c r="U18" s="41"/>
       <c r="AC18" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="AD18" s="44">
+      <c r="AD18" s="49">
         <v>54</v>
       </c>
-      <c r="AE18" s="44"/>
-      <c r="AF18" s="44"/>
-      <c r="AG18" s="44"/>
+      <c r="AE18" s="49"/>
+      <c r="AF18" s="49"/>
+      <c r="AG18" s="49"/>
       <c r="AN18" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="AO18" s="46">
+      <c r="AO18" s="41">
         <v>2.11</v>
       </c>
-      <c r="AP18" s="46"/>
-      <c r="AQ18" s="46"/>
-      <c r="AR18" s="46"/>
+      <c r="AP18" s="41"/>
+      <c r="AQ18" s="41"/>
+      <c r="AR18" s="41"/>
     </row>
     <row r="19" spans="1:44" ht="27.6" x14ac:dyDescent="0.3">
       <c r="F19" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="G19" s="45">
+      <c r="G19" s="50">
         <v>19500</v>
       </c>
-      <c r="H19" s="45"/>
-      <c r="I19" s="45"/>
-      <c r="J19" s="45"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="50"/>
+      <c r="J19" s="50"/>
       <c r="Q19" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="R19" s="46">
+      <c r="R19" s="41">
         <v>0.01</v>
       </c>
-      <c r="S19" s="46"/>
-      <c r="T19" s="46"/>
-      <c r="U19" s="46"/>
+      <c r="S19" s="41"/>
+      <c r="T19" s="41"/>
+      <c r="U19" s="41"/>
       <c r="AC19" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="AD19" s="45">
+      <c r="AD19" s="50">
         <v>19500</v>
       </c>
-      <c r="AE19" s="45"/>
-      <c r="AF19" s="45"/>
-      <c r="AG19" s="45"/>
+      <c r="AE19" s="50"/>
+      <c r="AF19" s="50"/>
+      <c r="AG19" s="50"/>
       <c r="AN19" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="AO19" s="46">
+      <c r="AO19" s="41">
         <v>0</v>
       </c>
-      <c r="AP19" s="46"/>
-      <c r="AQ19" s="46"/>
-      <c r="AR19" s="46"/>
+      <c r="AP19" s="41"/>
+      <c r="AQ19" s="41"/>
+      <c r="AR19" s="41"/>
     </row>
     <row r="20" spans="1:44" ht="61.2" x14ac:dyDescent="0.3">
       <c r="F20" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="G20" s="46" t="s">
+      <c r="G20" s="41" t="s">
         <v>249</v>
       </c>
-      <c r="H20" s="46"/>
-      <c r="I20" s="46"/>
-      <c r="J20" s="46"/>
+      <c r="H20" s="41"/>
+      <c r="I20" s="41"/>
+      <c r="J20" s="41"/>
       <c r="Q20" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="R20" s="46">
+      <c r="R20" s="41">
         <v>0</v>
       </c>
-      <c r="S20" s="46"/>
-      <c r="T20" s="46"/>
-      <c r="U20" s="46"/>
+      <c r="S20" s="41"/>
+      <c r="T20" s="41"/>
+      <c r="U20" s="41"/>
       <c r="AC20" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="AD20" s="46" t="s">
+      <c r="AD20" s="41" t="s">
         <v>250</v>
       </c>
-      <c r="AE20" s="46"/>
-      <c r="AF20" s="46"/>
-      <c r="AG20" s="46"/>
+      <c r="AE20" s="41"/>
+      <c r="AF20" s="41"/>
+      <c r="AG20" s="41"/>
       <c r="AN20" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="AO20" s="46">
+      <c r="AO20" s="41">
         <v>0</v>
       </c>
-      <c r="AP20" s="46"/>
-      <c r="AQ20" s="46"/>
-      <c r="AR20" s="46"/>
+      <c r="AP20" s="41"/>
+      <c r="AQ20" s="41"/>
+      <c r="AR20" s="41"/>
     </row>
     <row r="21" spans="1:44" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="F21" s="12" t="s">
@@ -8838,12 +8841,12 @@
       <c r="Q21" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="R21" s="44">
+      <c r="R21" s="49">
         <v>108</v>
       </c>
-      <c r="S21" s="44"/>
-      <c r="T21" s="44"/>
-      <c r="U21" s="44"/>
+      <c r="S21" s="49"/>
+      <c r="T21" s="49"/>
+      <c r="U21" s="49"/>
       <c r="AC21" s="12" t="s">
         <v>244</v>
       </c>
@@ -8853,12 +8856,12 @@
       <c r="AN21" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="AO21" s="44">
+      <c r="AO21" s="49">
         <v>108</v>
       </c>
-      <c r="AP21" s="44"/>
-      <c r="AQ21" s="44"/>
-      <c r="AR21" s="44"/>
+      <c r="AP21" s="49"/>
+      <c r="AQ21" s="49"/>
+      <c r="AR21" s="49"/>
     </row>
     <row r="22" spans="1:44" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F22" s="12" t="s">
@@ -8870,12 +8873,12 @@
       <c r="Q22" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="R22" s="45">
+      <c r="R22" s="50">
         <v>19500</v>
       </c>
-      <c r="S22" s="45"/>
-      <c r="T22" s="45"/>
-      <c r="U22" s="45"/>
+      <c r="S22" s="50"/>
+      <c r="T22" s="50"/>
+      <c r="U22" s="50"/>
       <c r="AC22" s="12" t="s">
         <v>252</v>
       </c>
@@ -8885,44 +8888,44 @@
       <c r="AN22" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="AO22" s="45">
+      <c r="AO22" s="50">
         <v>19500</v>
       </c>
-      <c r="AP22" s="45"/>
-      <c r="AQ22" s="45"/>
-      <c r="AR22" s="45"/>
+      <c r="AP22" s="50"/>
+      <c r="AQ22" s="50"/>
+      <c r="AR22" s="50"/>
     </row>
     <row r="23" spans="1:44" ht="33.6" x14ac:dyDescent="0.3">
       <c r="Q23" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="R23" s="46" t="s">
+      <c r="R23" s="41" t="s">
         <v>253</v>
       </c>
-      <c r="S23" s="46"/>
-      <c r="T23" s="46"/>
-      <c r="U23" s="46"/>
+      <c r="S23" s="41"/>
+      <c r="T23" s="41"/>
+      <c r="U23" s="41"/>
       <c r="AN23" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="AO23" s="46" t="s">
+      <c r="AO23" s="41" t="s">
         <v>254</v>
       </c>
-      <c r="AP23" s="46"/>
-      <c r="AQ23" s="46"/>
-      <c r="AR23" s="46"/>
+      <c r="AP23" s="41"/>
+      <c r="AQ23" s="41"/>
+      <c r="AR23" s="41"/>
     </row>
     <row r="24" spans="1:44" x14ac:dyDescent="0.3">
       <c r="Q24" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="R24" s="56">
+      <c r="R24" s="39">
         <v>2.1294360000000002E-3</v>
       </c>
       <c r="AN24" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="AO24" s="57">
+      <c r="AO24" s="40">
         <v>5.6517609999999998E-9</v>
       </c>
     </row>
@@ -8936,65 +8939,12 @@
       <c r="AN25" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="AO25" s="57">
+      <c r="AO25" s="40">
         <v>99.999989999999997</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="65">
-    <mergeCell ref="R22:U22"/>
-    <mergeCell ref="AO22:AR22"/>
-    <mergeCell ref="R23:U23"/>
-    <mergeCell ref="AO23:AR23"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="R20:U20"/>
-    <mergeCell ref="AD20:AG20"/>
-    <mergeCell ref="AO20:AR20"/>
-    <mergeCell ref="R21:U21"/>
-    <mergeCell ref="AO21:AR21"/>
-    <mergeCell ref="AN17:AR17"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="R18:U18"/>
-    <mergeCell ref="AD18:AG18"/>
-    <mergeCell ref="AO18:AR18"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="R19:U19"/>
-    <mergeCell ref="AD19:AG19"/>
-    <mergeCell ref="AO19:AR19"/>
-    <mergeCell ref="F14:J14"/>
-    <mergeCell ref="AC14:AG14"/>
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="G15:J15"/>
-    <mergeCell ref="AD15:AG15"/>
-    <mergeCell ref="G16:J16"/>
-    <mergeCell ref="AD16:AG16"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="Q17:U17"/>
-    <mergeCell ref="AD17:AG17"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="M12:O12"/>
-    <mergeCell ref="Y12:AA12"/>
-    <mergeCell ref="AJ12:AL12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="M13:O13"/>
-    <mergeCell ref="Y13:AA13"/>
-    <mergeCell ref="AJ13:AL13"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="M10:O10"/>
-    <mergeCell ref="Y10:AA10"/>
-    <mergeCell ref="AJ10:AL10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="Y11:AA11"/>
-    <mergeCell ref="AJ11:AL11"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="M8:O8"/>
-    <mergeCell ref="Y8:AA8"/>
-    <mergeCell ref="AJ8:AL8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="M9:O9"/>
-    <mergeCell ref="Y9:AA9"/>
-    <mergeCell ref="AJ9:AL9"/>
     <mergeCell ref="AI4:AL4"/>
     <mergeCell ref="AN4:AR4"/>
     <mergeCell ref="A7:D7"/>
@@ -9007,6 +8957,59 @@
     <mergeCell ref="R4:U4"/>
     <mergeCell ref="X4:AA4"/>
     <mergeCell ref="AC4:AG4"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="M8:O8"/>
+    <mergeCell ref="Y8:AA8"/>
+    <mergeCell ref="AJ8:AL8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="M9:O9"/>
+    <mergeCell ref="Y9:AA9"/>
+    <mergeCell ref="AJ9:AL9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="M10:O10"/>
+    <mergeCell ref="Y10:AA10"/>
+    <mergeCell ref="AJ10:AL10"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="Y11:AA11"/>
+    <mergeCell ref="AJ11:AL11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="M12:O12"/>
+    <mergeCell ref="Y12:AA12"/>
+    <mergeCell ref="AJ12:AL12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="M13:O13"/>
+    <mergeCell ref="Y13:AA13"/>
+    <mergeCell ref="AJ13:AL13"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="G15:J15"/>
+    <mergeCell ref="AD15:AG15"/>
+    <mergeCell ref="G16:J16"/>
+    <mergeCell ref="AD16:AG16"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="Q17:U17"/>
+    <mergeCell ref="AD17:AG17"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="R19:U19"/>
+    <mergeCell ref="AD19:AG19"/>
+    <mergeCell ref="AO19:AR19"/>
+    <mergeCell ref="F14:J14"/>
+    <mergeCell ref="AC14:AG14"/>
+    <mergeCell ref="AN17:AR17"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="R18:U18"/>
+    <mergeCell ref="AD18:AG18"/>
+    <mergeCell ref="AO18:AR18"/>
+    <mergeCell ref="R22:U22"/>
+    <mergeCell ref="AO22:AR22"/>
+    <mergeCell ref="R23:U23"/>
+    <mergeCell ref="AO23:AR23"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="R20:U20"/>
+    <mergeCell ref="AD20:AG20"/>
+    <mergeCell ref="AO20:AR20"/>
+    <mergeCell ref="R21:U21"/>
+    <mergeCell ref="AO21:AR21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>